<commit_message>
feat: add materials framework enhancements and UOM conversion support
- Added transaction processing mode using Source=filter
- Added MSSQL lookup provider support
- Added array lookup support
- Added Excel default value handling
- Added generic datetime conversion
- Fixed transaction template loading from selected format TemplateFile
- Excluded filter row from generated JSON processing
- Fixed MongoDB push when target array is null
- Verified Materials insert and UOM conversions update
</commit_message>
<xml_diff>
--- a/Templates/MaterialsSchema.xlsx
+++ b/Templates/MaterialsSchema.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitrepos\GMPPro20DataUpload\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\uploaddata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE999CB0-7800-4A10-A1F7-FA1A7075E044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B881B8-3648-46A6-B16E-9CBDC10EEEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9A0E982F-1D0A-437F-BDA7-ED9E8C087AEA}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="75">
   <si>
     <t>Property</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>settings</t>
+  </si>
+  <si>
+    <t>array</t>
   </si>
   <si>
     <t>materialFormattedName</t>
@@ -639,7 +642,7 @@
         <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -814,7 +817,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H9" t="s">
         <v>58</v>
@@ -891,7 +894,7 @@
         <v>6</v>
       </c>
       <c r="D13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
@@ -905,7 +908,7 @@
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
@@ -914,13 +917,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H14" t="s">
         <v>62</v>
       </c>
       <c r="I14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
@@ -1106,7 +1109,7 @@
         <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
         <v>6</v>
@@ -1115,13 +1118,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H23" t="s">
         <v>47</v>
       </c>
       <c r="I23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -1204,7 +1207,7 @@
         <v>38</v>
       </c>
       <c r="D27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" t="s">
         <v>42</v>
@@ -1247,10 +1250,10 @@
         <v>67</v>
       </c>
       <c r="C29" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="D29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
fix: stabilize upload framework after materials testing
- Added generic decimal datatype handling
- Added now() formula support
- Fixed optional lookup blank handling to set object fields as null
- Added template caching using existing cache service
- Added Test Database support for MongoDB and SQL connections
- Verified Materials, UOM Conversions, and optional usageUom behavior
</commit_message>
<xml_diff>
--- a/Templates/MaterialsSchema.xlsx
+++ b/Templates/MaterialsSchema.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\uploaddata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitrepos\GMPPro20DataUpload\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B881B8-3648-46A6-B16E-9CBDC10EEEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF81697C-7122-4C0D-9869-A10CCBC16790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9A0E982F-1D0A-437F-BDA7-ED9E8C087AEA}"/>
   </bookViews>
@@ -854,7 +854,7 @@
         <v>6</v>
       </c>
       <c r="D11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>

</xml_diff>